<commit_message>
updated check and cases
</commit_message>
<xml_diff>
--- a/Cases.xlsx
+++ b/Cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="235">
   <si>
     <t>ID</t>
   </si>
@@ -40,7 +40,7 @@
     <t>Наличие изображения на экране загрузки</t>
   </si>
   <si>
-    <t>Проверить  налилчие изображения на экране загрузки при запуске приложения</t>
+    <t xml:space="preserve"> Налилчие изображения на экране загрузки при запуске приложения</t>
   </si>
   <si>
     <t>Низкий</t>
@@ -58,7 +58,7 @@
     <t>Наличие цитаты на экране загрузки</t>
   </si>
   <si>
-    <t>Проверить  налилчие цитаты на экране загрузки при запуске приложения</t>
+    <t xml:space="preserve"> Налилчие цитаты на экране загрузки при запуске приложения</t>
   </si>
   <si>
     <t>На экране загрузки отображается цитата</t>
@@ -70,7 +70,7 @@
     <t>Работа прогресс-бара на экране загрузки</t>
   </si>
   <si>
-    <t>Проверить работу прогресс-бара на экране загрузки при запуске приложения</t>
+    <t>Работа прогресс-бара на экране загрузки при запуске приложения</t>
   </si>
   <si>
     <t>На экране загрузки заполняющийся прогресс-бар</t>
@@ -95,7 +95,7 @@
   </si>
   <si>
     <t>1) Открыть стартовую страницу приложения
-2) Проверить наличие полей "Login" и "Password"</t>
+2)   наличие полей "Login" и "Password"</t>
   </si>
   <si>
     <t>Поля "Login" и "Password" отображаются на экране</t>
@@ -127,7 +127,7 @@
     <t>Ввод некорректных данных (невалидный логин/пароль)</t>
   </si>
   <si>
-    <t>Проверить обработку неверных данных</t>
+    <t>Обработку неверных данных</t>
   </si>
   <si>
     <t>1) Ввести некорректные данные в поля логин и пароль
@@ -143,7 +143,7 @@
     <t>Вход с пустыми полями</t>
   </si>
   <si>
-    <t>Проверить поведение приложения при пустых полях</t>
+    <t>Авторизация при пустых полях</t>
   </si>
   <si>
     <t>Средний</t>
@@ -162,7 +162,7 @@
     <t>Поведение при неверном формате логина (например, с пробелами)</t>
   </si>
   <si>
-    <t>Проверить валидацию формата логина</t>
+    <t>Валидация формата логина</t>
   </si>
   <si>
     <t>1) Ввести логин с пробелами
@@ -175,7 +175,7 @@
     <t>Ввод символов в поле password (?%&amp;*)</t>
   </si>
   <si>
-    <t>Проверить корректность обработки специальных символов</t>
+    <t>Обработка специальных символов</t>
   </si>
   <si>
     <t>1) Ввести логин с символами (?%&amp;*)
@@ -188,7 +188,7 @@
     <t>Повторный запуск приложения после авторизации</t>
   </si>
   <si>
-    <t>Проверить, что пользователь остается залогиненым при перезапуске приложения</t>
+    <t>Пользователь остается залогиненым при перезапуске приложения</t>
   </si>
   <si>
     <t>1) Пользователь зарегистрирован
@@ -208,14 +208,14 @@
     <t>Наличие блока новостей</t>
   </si>
   <si>
-    <t>Убедиться, что на главной странице отображаются новости</t>
+    <t>На главной странице отображаются новости</t>
   </si>
   <si>
     <t xml:space="preserve">1) Пользователь авторизован
 </t>
   </si>
   <si>
-    <t>1) Проверить наличие блока новостей</t>
+    <t>1)   наличие блока новостей</t>
   </si>
   <si>
     <t>Блок новостей отображается</t>
@@ -227,7 +227,7 @@
     <t>Кнопка “ALL NEWS”</t>
   </si>
   <si>
-    <t>Учебиться, что кнопка "ALL NEWS" кликабельная и переносит на страницу новостей</t>
+    <t>Кнопка "ALL NEWS" кликабельная и переносит на страницу новостей</t>
   </si>
   <si>
     <t>1) Пользователь авторизован
@@ -300,7 +300,7 @@
     <t>Работа фильтра новостей</t>
   </si>
   <si>
-    <t>Проверить фильтрацию новостей по категориям, дате публикации</t>
+    <t>Фильтрация новостей по категориям, дате публикации</t>
   </si>
   <si>
     <t>1) Пользователь авторизован
@@ -328,7 +328,7 @@
 </t>
   </si>
   <si>
-    <t>Проверить возможность отменить выбранный фильтр</t>
+    <t>Возможность отменить выбранный фильтр</t>
   </si>
   <si>
     <t>1) Тапнуть по списку категорий
@@ -350,7 +350,7 @@
     <t>Фильтрация по дате добавления новости</t>
   </si>
   <si>
-    <t>Проверить работу фильтрации по дате добавления новостей</t>
+    <t>Фильтрация по дате добавления новостей</t>
   </si>
   <si>
     <t>1) Тапнуть по кнопке фильтрации по датей добавления (стрелки вверх/вниз)</t>
@@ -365,7 +365,7 @@
     <t>Кнопка "REFRESH"</t>
   </si>
   <si>
-    <t>Проверить работу кнопки "REFRESH" при отсутствии новостей</t>
+    <t>Кнопка "REFRESH" при отсутствии новостей</t>
   </si>
   <si>
     <t>1) Тапнуть по кнопке "REFRESH"</t>
@@ -380,7 +380,7 @@
     <t>Страница добавления новостей</t>
   </si>
   <si>
-    <t>Проверка, что открывается страница добавления новости и есть все необходимые поля</t>
+    <t>Страница добавления новости открывается и есть все необходимые поля</t>
   </si>
   <si>
     <t>1) Пользователь авторизован
@@ -399,7 +399,7 @@
     <t>Категории при добавлении новостей</t>
   </si>
   <si>
-    <t>Проверить, что новость выкладывается в той категории, которую указал пользователь</t>
+    <t>Новость выкладывается в той категории, которую указал пользователь</t>
   </si>
   <si>
     <t>1) Пользователь авторизован
@@ -420,7 +420,7 @@
     <t>Пустое поле "Title"</t>
   </si>
   <si>
-    <t>Проверить, что при пустом поле "Title", новость не опубликуется</t>
+    <t>При пустом поле "Title", новость не опубликуется</t>
   </si>
   <si>
     <t>1) Заполнить поля корректными данными
@@ -436,12 +436,12 @@
     <t xml:space="preserve">Новость публикуется с учетом даты указанной в поле "Publication date" </t>
   </si>
   <si>
-    <t>Проверить что новость публикуется в дату, которая указана в поле "Publication date"</t>
+    <t>Новость публикуется в дату, которая указана в поле "Publication date"</t>
   </si>
   <si>
     <t>1) Заполнить поля корректными данными
 2) Установить нужную дату
-3) Проверить опубликовалась ли новость в указанную дату</t>
+3)   опубликовалась ли новость в указанную дату</t>
   </si>
   <si>
     <t>Новость публикуется в указанную дату</t>
@@ -453,12 +453,12 @@
     <t xml:space="preserve">Новость публикуется с учетом времени указанном в поле "Time" </t>
   </si>
   <si>
-    <t>Проверить что новость публикуется во время, указанное в поле "Time"</t>
+    <t>Новость публикуется во время, указанное в поле "Time"</t>
   </si>
   <si>
     <t>1) Заполнить поля корректными данными
 2) Установить нужное время
-3) Проверить опубликовалась ли новость в указанное время</t>
+3)   опубликовалась ли новость в указанное время</t>
   </si>
   <si>
     <t>Новость публикуется в указанное время</t>
@@ -470,7 +470,7 @@
     <t>Заполнение поля "Time" вручную</t>
   </si>
   <si>
-    <t>Проверить, что можно ввести только корректный формат времени</t>
+    <t>Вводится только корректный формат времени</t>
   </si>
   <si>
     <t>1) Заполнить поля корректными данными
@@ -488,7 +488,7 @@
     <t>Пустое поле "Description"</t>
   </si>
   <si>
-    <t>Проверить, что при пустом поле "Description" новость не опубликуется</t>
+    <t>При пустом поле "Description" новость не опубликуется</t>
   </si>
   <si>
     <t>1) Заполнить поля корректными данными
@@ -501,7 +501,7 @@
     <t xml:space="preserve">Ползунок "Active" </t>
   </si>
   <si>
-    <t>Проверить, что можно поменять состояние ползунка с "Active" на "Iactive" и наоборот</t>
+    <t xml:space="preserve"> Состояние ползунка меняется с "Active" на "Iactive" и наоборот</t>
   </si>
   <si>
     <t>1) Заполнить поля корректными данными
@@ -520,7 +520,7 @@
     <t>Работа кнопки "Cancel"</t>
   </si>
   <si>
-    <t>Проверить, что с помощью кнопки "Cancel" можно отменить публикацию новости</t>
+    <t>Кнопка "Cancel" отменяет публикацию новости</t>
   </si>
   <si>
     <t>1) Тапнуть по кнопке "Cancel"
@@ -536,7 +536,7 @@
     <t>Работа кнопки "Cancel" с запоненными данными</t>
   </si>
   <si>
-    <t>Проверить, что с помощью кнопки "Cancel" можно отменить публикацию новости даже если данные уже заполнены</t>
+    <t>Кнопка "Cancel" отменяет публикацию новости даже если данные уже заполнены</t>
   </si>
   <si>
     <t>1) Заполнить поля корректными данными
@@ -547,14 +547,11 @@
     <t>Публикация новости</t>
   </si>
   <si>
-    <t>Проверить, что новость публикуется</t>
+    <t>Новость публикуется</t>
   </si>
   <si>
     <t>1) Заполнить поля корректными данными
 2) Тапнуть по кнопке "Save"</t>
-  </si>
-  <si>
-    <t>Новость публикуется</t>
   </si>
   <si>
     <t>Модули NEWS и ADDNEWS будет невохможно автоматизировать т.к на данный момент функционал добавления новостей и работа фильтров не реализованы</t>
@@ -566,7 +563,7 @@
     <t>Переход на страницу "About"</t>
   </si>
   <si>
-    <t>Проверка, что страницы "About" доступна</t>
+    <t>Страница "About" доступна</t>
   </si>
   <si>
     <t>1) Пользователь авторизован
@@ -586,7 +583,7 @@
     <t>Отображение версии приложения</t>
   </si>
   <si>
-    <t>Проверить, версия приложения отображается</t>
+    <t>Версия приложения отображается</t>
   </si>
   <si>
     <t>1) Пользователь авторизован
@@ -605,7 +602,7 @@
     <t>Ссылка "Privacy Policy"</t>
   </si>
   <si>
-    <t>Проверить, что ссылка видима и работает</t>
+    <t>Ссылка видима и работает</t>
   </si>
   <si>
     <t>1) Обратить внимание на текст "Privacy Policy:"
@@ -631,7 +628,7 @@
     <t>Кнопка меню присутствует и кликабельна</t>
   </si>
   <si>
-    <t>Проверить, что кнопка меню (три полоски в левом верхнем углу на главном экране) есть и на нее можно кликнуть</t>
+    <t>Кнопка меню (три полоски в левом верхнем углу на главном экране) есть и на нее можно кликнуть</t>
   </si>
   <si>
     <t xml:space="preserve">1) Тапнуть по кнопке меню </t>
@@ -646,7 +643,7 @@
     <t>Переход на страницу "News"</t>
   </si>
   <si>
-    <t>Проверить, что есть возможность перейти на страницу "News", через меню</t>
+    <t>Есть возможность перейти на страницу "News", через меню</t>
   </si>
   <si>
     <t>1) Тапнуть по кнопке меню
@@ -662,7 +659,7 @@
     <t>Переход между страницами через меню</t>
   </si>
   <si>
-    <t>Проверить, что есть возможность переходить между страницами через меню</t>
+    <t>Возможно переходить между страницами через меню</t>
   </si>
   <si>
     <t>1) Пользователь авторизован
@@ -686,7 +683,7 @@
     <t>Закрытие меню</t>
   </si>
   <si>
-    <t>Проверить, что меню можно закрыть тапом по любой области экрана</t>
+    <t>Меню закрывается тапом по любой области экрана</t>
   </si>
   <si>
     <t>1) Открыто меню</t>
@@ -704,7 +701,7 @@
     <t>Переход на страницу "Love os all"</t>
   </si>
   <si>
-    <t>Проверить, что есть возможность перейти на страницу "Love is all" из страниц "Main", "Control panel", "News"</t>
+    <t>Есть переход на страницу "Love is all" из страниц "Main", "Control panel", "News"</t>
   </si>
   <si>
     <t>1) Пользователь авторизован
@@ -718,10 +715,13 @@
     <t>При наличии иконки бабочки на экране, при тапе на нее, совершается переход на страницу "Love is all" из страниц "Main", "Control panel", "News"</t>
   </si>
   <si>
+    <t>QUOTE-02</t>
+  </si>
+  <si>
     <t xml:space="preserve">Отображение списки цитат </t>
   </si>
   <si>
-    <t>Проверить, что цитаты отображаются на странице "Love is all"</t>
+    <t>Цитаты отображаются на странице "Love is all"</t>
   </si>
   <si>
     <t>1) Пользователь авторизован
@@ -734,10 +734,13 @@
     <t>На странице "Love is all" отображаются цитаты</t>
   </si>
   <si>
+    <t>QUOTE-03</t>
+  </si>
+  <si>
     <t>Раскрытие отображаемых цитат</t>
   </si>
   <si>
-    <t>Проверить, что цитаты можно раскрыть при тапе на них</t>
+    <t>Цитаты можно раскрыть при тапе на них</t>
   </si>
   <si>
     <t>1) Тапнуть по одной из отображаемых цитат</t>
@@ -746,10 +749,13 @@
     <t>Цитата раскрывается и можно прочитать ее продолжение</t>
   </si>
   <si>
+    <t>QUOTE-04</t>
+  </si>
+  <si>
     <t>Закрытие развернутых цитат</t>
   </si>
   <si>
-    <t>Проверить, что цитаты можно закрыть при повторном тапе по ним</t>
+    <t>Цитаты можно закрыть при повторном тапе по ним</t>
   </si>
   <si>
     <t>1) Пользователь авторизован
@@ -769,7 +775,7 @@
     <t>Кнопка выхода из аккаунта</t>
   </si>
   <si>
-    <t>Проверить наличие и работу кнопки для выхода из аккаунта</t>
+    <t>При нажатии на кнопку для выхода из аккауньа происходит выход из аккаунта</t>
   </si>
   <si>
     <t>1) Пользователь авторизован</t>
@@ -2587,7 +2593,7 @@
         <v>162</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
@@ -2611,7 +2617,7 @@
     </row>
     <row r="38">
       <c r="A38" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
@@ -2669,25 +2675,25 @@
     </row>
     <row r="40">
       <c r="A40" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="B40" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="C40" s="8" t="s">
         <v>166</v>
-      </c>
-      <c r="C40" s="8" t="s">
-        <v>167</v>
       </c>
       <c r="D40" s="12" t="s">
         <v>25</v>
       </c>
       <c r="E40" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="F40" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="F40" s="8" t="s">
+      <c r="G40" s="8" t="s">
         <v>169</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>170</v>
       </c>
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
@@ -2711,25 +2717,25 @@
     </row>
     <row r="41">
       <c r="A41" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="B41" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="C41" s="8" t="s">
         <v>172</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>173</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>10</v>
       </c>
       <c r="E41" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="F41" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="F41" s="8" t="s">
+      <c r="G41" s="8" t="s">
         <v>175</v>
-      </c>
-      <c r="G41" s="8" t="s">
-        <v>176</v>
       </c>
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
@@ -2753,25 +2759,25 @@
     </row>
     <row r="42">
       <c r="A42" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B42" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="C42" s="8" t="s">
         <v>178</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>179</v>
       </c>
       <c r="D42" s="14" t="s">
         <v>43</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F42" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="G42" s="8" t="s">
         <v>180</v>
-      </c>
-      <c r="G42" s="8" t="s">
-        <v>181</v>
       </c>
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
@@ -2795,25 +2801,25 @@
     </row>
     <row r="43">
       <c r="A43" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B43" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="B43" s="8" t="s">
-        <v>183</v>
-      </c>
       <c r="C43" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D43" s="14" t="s">
         <v>43</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>
@@ -2858,25 +2864,25 @@
     </row>
     <row r="45">
       <c r="A45" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B45" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="C45" s="8" t="s">
         <v>186</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>187</v>
       </c>
       <c r="D45" s="12" t="s">
         <v>25</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F45" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="G45" s="8" t="s">
         <v>188</v>
-      </c>
-      <c r="G45" s="8" t="s">
-        <v>189</v>
       </c>
       <c r="H45" s="7"/>
       <c r="I45" s="7"/>
@@ -2900,25 +2906,25 @@
     </row>
     <row r="46">
       <c r="A46" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B46" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="B46" s="8" t="s">
+      <c r="C46" s="8" t="s">
         <v>191</v>
-      </c>
-      <c r="C46" s="8" t="s">
-        <v>192</v>
       </c>
       <c r="D46" s="14" t="s">
         <v>43</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F46" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="G46" s="8" t="s">
         <v>193</v>
-      </c>
-      <c r="G46" s="8" t="s">
-        <v>194</v>
       </c>
       <c r="H46" s="7"/>
       <c r="I46" s="7"/>
@@ -2942,25 +2948,25 @@
     </row>
     <row r="47">
       <c r="A47" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="B47" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="B47" s="8" t="s">
+      <c r="C47" s="8" t="s">
         <v>196</v>
-      </c>
-      <c r="C47" s="8" t="s">
-        <v>197</v>
       </c>
       <c r="D47" s="14" t="s">
         <v>43</v>
       </c>
       <c r="E47" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="F47" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="F47" s="8" t="s">
+      <c r="G47" s="8" t="s">
         <v>199</v>
-      </c>
-      <c r="G47" s="8" t="s">
-        <v>200</v>
       </c>
       <c r="H47" s="7"/>
       <c r="I47" s="7"/>
@@ -2984,25 +2990,25 @@
     </row>
     <row r="48">
       <c r="A48" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="B48" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="B48" s="8" t="s">
+      <c r="C48" s="8" t="s">
         <v>202</v>
-      </c>
-      <c r="C48" s="8" t="s">
-        <v>203</v>
       </c>
       <c r="D48" s="9" t="s">
         <v>10</v>
       </c>
       <c r="E48" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="F48" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="F48" s="8" t="s">
+      <c r="G48" s="8" t="s">
         <v>205</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>206</v>
       </c>
       <c r="H48" s="7"/>
       <c r="I48" s="7"/>
@@ -3054,25 +3060,25 @@
     </row>
     <row r="50">
       <c r="A50" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="B50" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="C50" s="8" t="s">
         <v>208</v>
-      </c>
-      <c r="C50" s="8" t="s">
-        <v>209</v>
       </c>
       <c r="D50" s="14" t="s">
         <v>43</v>
       </c>
       <c r="E50" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="F50" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="F50" s="8" t="s">
+      <c r="G50" s="8" t="s">
         <v>211</v>
-      </c>
-      <c r="G50" s="8" t="s">
-        <v>212</v>
       </c>
       <c r="H50" s="7"/>
       <c r="I50" s="7"/>
@@ -3096,7 +3102,7 @@
     </row>
     <row r="51">
       <c r="A51" s="8" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B51" s="8" t="s">
         <v>213</v>
@@ -3138,13 +3144,13 @@
     </row>
     <row r="52">
       <c r="A52" s="8" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D52" s="12" t="s">
         <v>25</v>
@@ -3153,10 +3159,10 @@
         <v>215</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H52" s="7"/>
       <c r="I52" s="7"/>
@@ -3180,25 +3186,25 @@
     </row>
     <row r="53">
       <c r="A53" s="8" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D53" s="9" t="s">
         <v>10</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="H53" s="7"/>
       <c r="I53" s="7"/>
@@ -3250,25 +3256,25 @@
     </row>
     <row r="55">
       <c r="A55" s="8" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D55" s="12" t="s">
         <v>25</v>
       </c>
       <c r="E55" s="19" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F55" s="19" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="H55" s="7"/>
       <c r="I55" s="7"/>

</xml_diff>